<commit_message>
Latest update for the PoR case study
</commit_message>
<xml_diff>
--- a/inventories/lci-open-prom.xlsx
+++ b/inventories/lci-open-prom.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\terlouw_t\Documents\Projects\TRANSIENCE\lca_port_of_rotterdam\inventories\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\terlouw_t\Documents\Projects\TRANSIENCE\lca_transience\inventories\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9FEC5DB-D7DF-4248-AA15-51A4A084F598}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79DD8816-9578-48AC-A195-17850C86110D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28740" yWindow="-21600" windowWidth="26010" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="33885" yWindow="-21600" windowWidth="20865" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="lci" sheetId="9" r:id="rId1"/>

</xml_diff>

<commit_message>
Larger update, to also show steel implementation test from ITOM
</commit_message>
<xml_diff>
--- a/inventories/lci-open-prom.xlsx
+++ b/inventories/lci-open-prom.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\terlouw_t\Documents\Projects\TRANSIENCE\lca_transience\inventories\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79DD8816-9578-48AC-A195-17850C86110D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60E4FBED-73FA-4634-9D01-270552DE9440}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="33885" yWindow="-21600" windowWidth="20865" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28740" yWindow="-21600" windowWidth="26010" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="lci" sheetId="9" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10052" uniqueCount="615">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10052" uniqueCount="618">
   <si>
     <t>Activity</t>
   </si>
@@ -1889,6 +1889,15 @@
   </si>
   <si>
     <t>light fuel oil, burned in industrial furnace</t>
+  </si>
+  <si>
+    <t>fuel tank, compressed hydrogen gas, 700bar, with HDPE liner, carculator passenger car 2020</t>
+  </si>
+  <si>
+    <t>hydrogen tank</t>
+  </si>
+  <si>
+    <t>electricity production, photovoltaic, 3kWp slanted-roof installation, multi-Si, laminated, integrated</t>
   </si>
 </sst>
 </file>
@@ -4504,7 +4513,7 @@
     </row>
     <row r="129" spans="1:11">
       <c r="A129" t="s">
-        <v>503</v>
+        <v>617</v>
       </c>
       <c r="B129" s="3">
         <v>1</v>
@@ -5065,7 +5074,7 @@
     </row>
     <row r="170" spans="1:11">
       <c r="A170" t="s">
-        <v>399</v>
+        <v>615</v>
       </c>
       <c r="B170">
         <f>802/1000000/10.95</f>
@@ -5081,7 +5090,7 @@
         <v>18</v>
       </c>
       <c r="G170" t="s">
-        <v>398</v>
+        <v>616</v>
       </c>
       <c r="H170">
         <v>5</v>

</xml_diff>